<commit_message>
tehnohaus - insizew update
</commit_message>
<xml_diff>
--- a/Javascript Vanilla/tehnohaus.mk/katalozi/Kategorii od katalozi.xlsx
+++ b/Javascript Vanilla/tehnohaus.mk/katalozi/Kategorii od katalozi.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="667" activeTab="13"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="667" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="CetaForm" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,6 @@
     <sheet name="Altec" sheetId="10" r:id="rId11"/>
     <sheet name="Stubai" sheetId="11" r:id="rId12"/>
     <sheet name="HFS" sheetId="12" r:id="rId13"/>
-    <sheet name="Insize (2)" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="453">
   <si>
     <t>TOOL CONTAINERS AND ASSORTMENTS</t>
   </si>
@@ -1348,15 +1347,9 @@
     <t>Рачни и машински либели</t>
   </si>
   <si>
-    <t>Линеари, дигитални индикатори, воздушни мерила, тестери за истекување на воздух, ласерски скен микрометри, спектрометри, преднаместувачи на алати</t>
-  </si>
-  <si>
     <t>Разновидни детектори</t>
   </si>
   <si>
-    <t>(cmm) координатни мерни машини</t>
-  </si>
-  <si>
     <t>Профил проектори, системи за брзо мерење, визуелни мерни системи</t>
   </si>
   <si>
@@ -1399,64 +1392,10 @@
     <t>Мерач на спреј на сол, комори за температура и влажност</t>
   </si>
   <si>
-    <t>Insize 1. Експорт на податоци и софтвер</t>
-  </si>
-  <si>
-    <t>Insize 10. Мерачи на косини</t>
-  </si>
-  <si>
-    <t>Insize 2. Шублери</t>
-  </si>
-  <si>
-    <t>Insize 3. Мерачи на длабочина</t>
-  </si>
-  <si>
-    <t>Insize 4. Мерачи на висина</t>
-  </si>
-  <si>
-    <t>Insize 5. Компаратори</t>
-  </si>
-  <si>
-    <t>Insize 6. Микрометри</t>
-  </si>
-  <si>
-    <t>Insize 7. Мерачи на дијаметар и опсег на отвори</t>
-  </si>
-  <si>
-    <t>Insize 8. Мерачи на радиус на лак</t>
-  </si>
-  <si>
-    <t>Insize 9. Мерачи на жлебови за клучеви</t>
-  </si>
-  <si>
-    <t>Insize 1. DATA OUTPUT AND SOFTWARE.pdf</t>
-  </si>
-  <si>
-    <t>Insize 2. CALIPERS.pdf</t>
-  </si>
-  <si>
-    <t>Insize 3. DEPTH MEASUREMENT.pdf</t>
-  </si>
-  <si>
-    <t>Insize 4. HEIGHT MEASUREMENT.pdf</t>
-  </si>
-  <si>
-    <t>Insize 5. COMPARISON INSTRUMENTS.pdf</t>
-  </si>
-  <si>
-    <t>Insize 6. MICROMETERS.pdf</t>
-  </si>
-  <si>
-    <t>Insize 7. BORE DIAMETER, CIRCUMFERENCE MEASUREMENT.pdf</t>
-  </si>
-  <si>
-    <t>Insize 8. ARC RADIUS MEASUREMENT.pdf</t>
-  </si>
-  <si>
-    <t>Insize 9. KEYWAY MEASUREMENT.pdf</t>
-  </si>
-  <si>
-    <t>Insize 10. CHAMFER MEASUREMENT.pdf</t>
+    <t>Линеари, дигитални индикатори, воздушни мерила, тестери за истекување на воздух, ласерски скен микрометри, спектрометри</t>
+  </si>
+  <si>
+    <t>CMM - координатни мерни машини</t>
   </si>
 </sst>
 </file>
@@ -2945,137 +2884,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>463</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>453</v>
-      </c>
-      <c r="C2" t="str">
-        <f>"Rename-Item -LiteralPath '"&amp;A2&amp;"' -NewName """&amp;SUBSTITUTE(B2,"""","`"") &amp; """"")</f>
-        <v>Rename-Item -LiteralPath 'Insize 1. DATA OUTPUT AND SOFTWARE.pdf' -NewName "Insize 1. Експорт на податоци и софтвер</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>464</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>455</v>
-      </c>
-      <c r="C3" t="str">
-        <f t="shared" ref="C3:C11" si="0">"Rename-Item -LiteralPath '"&amp;A3&amp;"' -NewName """&amp;SUBSTITUTE(B3,"""","`"") &amp; """"")</f>
-        <v>Rename-Item -LiteralPath 'Insize 2. CALIPERS.pdf' -NewName "Insize 2. Шублери</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>465</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="C4" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 3. DEPTH MEASUREMENT.pdf' -NewName "Insize 3. Мерачи на длабочина</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>466</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>457</v>
-      </c>
-      <c r="C5" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 4. HEIGHT MEASUREMENT.pdf' -NewName "Insize 4. Мерачи на висина</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>467</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>458</v>
-      </c>
-      <c r="C6" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 5. COMPARISON INSTRUMENTS.pdf' -NewName "Insize 5. Компаратори</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>468</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>459</v>
-      </c>
-      <c r="C7" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 6. MICROMETERS.pdf' -NewName "Insize 6. Микрометри</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>469</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>460</v>
-      </c>
-      <c r="C8" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 7. BORE DIAMETER, CIRCUMFERENCE MEASUREMENT.pdf' -NewName "Insize 7. Мерачи на дијаметар и опсег на отвори</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>470</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>461</v>
-      </c>
-      <c r="C9" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 8. ARC RADIUS MEASUREMENT.pdf' -NewName "Insize 8. Мерачи на радиус на лак</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>471</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>462</v>
-      </c>
-      <c r="C10" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 9. KEYWAY MEASUREMENT.pdf' -NewName "Insize 9. Мерачи на жлебови за клучеви</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>472</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>454</v>
-      </c>
-      <c r="C11" t="str">
-        <f t="shared" si="0"/>
-        <v>Rename-Item -LiteralPath 'Insize 10. CHAMFER MEASUREMENT.pdf' -NewName "Insize 10. Мерачи на косини</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q21"/>
@@ -3510,419 +3318,419 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>82</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>71</v>
       </c>
-      <c r="O4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>83</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>84</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>85</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
         <v>72</v>
       </c>
-      <c r="O8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
         <v>86</v>
       </c>
-      <c r="O9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
         <v>87</v>
       </c>
-      <c r="O10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
         <v>88</v>
       </c>
-      <c r="O11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" t="s">
         <v>89</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>90</v>
       </c>
-      <c r="O13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" t="s">
         <v>73</v>
       </c>
-      <c r="O14" s="4" t="s">
+      <c r="G14" s="4" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" t="s">
         <v>91</v>
       </c>
-      <c r="O15" s="4" t="s">
+      <c r="G15" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" t="s">
         <v>74</v>
       </c>
-      <c r="O16" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>92</v>
       </c>
-      <c r="O17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18" t="s">
         <v>93</v>
       </c>
-      <c r="O18" s="4" t="s">
+      <c r="G18" s="4" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19" t="s">
         <v>75</v>
       </c>
-      <c r="O19" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20" t="s">
         <v>76</v>
       </c>
-      <c r="O20" s="4" t="s">
+      <c r="G20" s="4" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21" t="s">
         <v>94</v>
       </c>
-      <c r="O21" s="4" t="s">
+      <c r="G21" s="4" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>80</v>
       </c>
-      <c r="O22" s="4" t="s">
+      <c r="G22" s="4" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>183</v>
       </c>
-      <c r="O23" s="4" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G23" s="4" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>95</v>
       </c>
-      <c r="O24" s="4" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G24" s="4" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
       <c r="B25" t="s">
         <v>96</v>
       </c>
-      <c r="O25" s="4" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G25" s="4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
       <c r="B26" t="s">
         <v>97</v>
       </c>
-      <c r="O26" s="4" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G26" s="4" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
       <c r="B27" t="s">
         <v>98</v>
       </c>
-      <c r="O27" s="4" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G27" s="4" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
       <c r="B28" t="s">
         <v>99</v>
       </c>
-      <c r="O28" s="4" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G28" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>27</v>
       </c>
       <c r="B29" t="s">
         <v>100</v>
       </c>
-      <c r="O29" s="4" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G29" s="4" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
       <c r="B30" t="s">
         <v>79</v>
       </c>
-      <c r="O30" s="4" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G30" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
       <c r="B31" t="s">
         <v>101</v>
       </c>
-      <c r="O31" s="4" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G31" s="4" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
       <c r="B32" t="s">
         <v>102</v>
       </c>
-      <c r="O32" s="4" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G32" s="4" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>31</v>
       </c>
       <c r="B33" t="s">
         <v>78</v>
       </c>
-      <c r="O33" s="4" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G33" s="4" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>32</v>
       </c>
       <c r="B34" t="s">
         <v>81</v>
       </c>
-      <c r="O34" s="4" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G34" s="4" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>33</v>
       </c>
       <c r="B35" t="s">
         <v>103</v>
       </c>
-      <c r="O35" s="4" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G35" s="4" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>34</v>
       </c>
       <c r="B36" t="s">
         <v>104</v>
       </c>
-      <c r="O36" s="4" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G36" s="4" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>35</v>
       </c>
       <c r="B37" t="s">
         <v>105</v>
       </c>
-      <c r="O37" s="4" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G37" s="4" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>36</v>
       </c>
       <c r="B38" t="s">
         <v>77</v>
       </c>
-      <c r="O38" s="4" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="G38" s="4" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>37</v>
       </c>
       <c r="B39" t="s">
         <v>106</v>
       </c>
-      <c r="O39" s="4" t="s">
-        <v>452</v>
+      <c r="G39" s="4" t="s">
+        <v>450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>